<commit_message>
Handle the native success alert on Register/Add User, use Rachana in Register test data
The site shows a native "User registered successfully." alert after a
successful submit, which the reference PDF doesn't account for - any
further WebDriver command threw UnhandledAlertException. Accept the alert
(if present) right after clicking submit in RegisterBL and AddUserBL.
</commit_message>
<xml_diff>
--- a/Aug26_And_Aug27_SeleniumAutomationProject_ExcelAndProperties/src/test/resources/TestData.xlsx
+++ b/Aug26_And_Aug27_SeleniumAutomationProject_ExcelAndProperties/src/test/resources/TestData.xlsx
@@ -50,15 +50,6 @@
     <t>Mobile</t>
   </si>
   <si>
-    <t>Rahul</t>
-  </si>
-  <si>
-    <t>rahul@gmail.com</t>
-  </si>
-  <si>
-    <t>Rahul@123</t>
-  </si>
-  <si>
     <t>abc</t>
   </si>
   <si>
@@ -93,6 +84,15 @@
   </si>
   <si>
     <t>amit</t>
+  </si>
+  <si>
+    <t>Rachana</t>
+  </si>
+  <si>
+    <t>rachana@gmail.com</t>
+  </si>
+  <si>
+    <t>Rachana@123</t>
   </si>
 </sst>
 </file>
@@ -520,16 +520,16 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C2">
         <v>9876543210</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -540,7 +540,7 @@
         <v>123</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -558,7 +558,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>9</v>
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -584,25 +584,25 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C2">
         <v>9876543210</v>
       </c>
       <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -613,7 +613,7 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>